<commit_message>
Add comprehensive system-wide stress tests (37 tests, 467 total)
Stress tests cover all 5 phases at scale: 50K equity-cash netting,
600-position derivatives MTM, SPAN across 15 underlyings, 100 debt
DvP-I settlements, 20-node CM hierarchy, SGF waterfall edge cases,
cross-module integration chains, and boundary conditions.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/generated/settlement_report.xlsx
+++ b/data/generated/settlement_report.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-21 11:47</t>
+          <t>2026-06-23 16:51</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>000f614f-1d4...</t>
+          <t>49407354-33e...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>942150a6-2d4...</t>
+          <t>15f3b0ba-78c...</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -753,10 +753,10 @@
         <v>381663.84</v>
       </c>
       <c r="F2" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G2" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -771,12 +771,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>666317a1-411...</t>
+          <t>9af5d587-8d8...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>92133f1b-306...</t>
+          <t>0cccde10-ee6...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -793,10 +793,10 @@
         <v>9690493.68</v>
       </c>
       <c r="F3" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G3" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -811,12 +811,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>bc5e3955-b0b...</t>
+          <t>254dad86-f0f...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>ca8e2fd1-4d4...</t>
+          <t>dcfe1c32-671...</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -833,10 +833,10 @@
         <v>299960.95</v>
       </c>
       <c r="F4" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G4" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -851,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>f979de19-295...</t>
+          <t>65f94147-1c5...</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>91da00c1-f5c...</t>
+          <t>50aee2df-404...</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -873,10 +873,10 @@
         <v>791189.8100000001</v>
       </c>
       <c r="F5" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G5" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -891,12 +891,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>7d411d9f-e26...</t>
+          <t>4633a7a1-6e8...</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9dafce4d-846...</t>
+          <t>d3ab5f27-f61...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -913,10 +913,10 @@
         <v>64504.72</v>
       </c>
       <c r="F6" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G6" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -931,12 +931,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>659b982d-af0...</t>
+          <t>98a6268e-99d...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2f0ac22b-8d8...</t>
+          <t>32ac8893-1e6...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -953,10 +953,10 @@
         <v>273807.91</v>
       </c>
       <c r="F7" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G7" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -971,12 +971,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>42d3969f-33b...</t>
+          <t>f0232e8f-bbe...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2c4f60fb-938...</t>
+          <t>32ac5fe1-dc9...</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -993,10 +993,10 @@
         <v>1083230.88</v>
       </c>
       <c r="F8" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G8" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1011,12 +1011,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>0f7423d9-90c...</t>
+          <t>ce9f28fd-8fd...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>b8a3cf86-ea9...</t>
+          <t>6193d5a3-5e7...</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1033,10 +1033,10 @@
         <v>1547871.14</v>
       </c>
       <c r="F9" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G9" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1051,12 +1051,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>fe1e4bd4-bb8...</t>
+          <t>00d1e095-4f9...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>d9a5c764-8d1...</t>
+          <t>267b501d-9d8...</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1073,10 +1073,10 @@
         <v>29074.73</v>
       </c>
       <c r="F10" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G10" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1091,12 +1091,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>24e1260b-f03...</t>
+          <t>83a85f0b-ced...</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>bff17479-e29...</t>
+          <t>413dadeb-637...</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1113,10 +1113,10 @@
         <v>1713.96</v>
       </c>
       <c r="F11" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G11" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>b7437ccb-c17...</t>
+          <t>82498ff5-70b...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>c1507161-b90...</t>
+          <t>92b7fc01-bd6...</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1153,10 +1153,10 @@
         <v>68693.5</v>
       </c>
       <c r="F12" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G12" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1171,12 +1171,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>f728400a-35d...</t>
+          <t>4b987458-5a9...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>24363809-161...</t>
+          <t>a4e9c383-dc5...</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1193,10 +1193,10 @@
         <v>11915.98</v>
       </c>
       <c r="F13" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G13" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1211,12 +1211,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>3d9547cf-14b...</t>
+          <t>a3f87049-6f4...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>e34bdf46-ea7...</t>
+          <t>0dda435d-f20...</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1233,10 +1233,10 @@
         <v>356892.18</v>
       </c>
       <c r="F14" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G14" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1251,12 +1251,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>6ed50332-dbe...</t>
+          <t>0fa1d430-7f7...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7763074b-559...</t>
+          <t>08375d86-bad...</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1273,10 +1273,10 @@
         <v>24294.34</v>
       </c>
       <c r="F15" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G15" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1291,12 +1291,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>820600f7-416...</t>
+          <t>89311f79-7ed...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>6d0d7100-24a...</t>
+          <t>ae531cee-f05...</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1313,10 +1313,10 @@
         <v>243.43</v>
       </c>
       <c r="F16" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G16" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1331,12 +1331,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>a47fd18a-49f...</t>
+          <t>812c1fe9-9e0...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ad32683e-4bd...</t>
+          <t>0e980820-06d...</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1353,10 +1353,10 @@
         <v>479876.4</v>
       </c>
       <c r="F17" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G17" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1371,12 +1371,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>71e6cf93-e06...</t>
+          <t>72f6de25-78e...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>984197fc-bfd...</t>
+          <t>ee0bcbb0-c99...</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1393,10 +1393,10 @@
         <v>163612.58</v>
       </c>
       <c r="F18" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G18" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1411,12 +1411,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>a3c6b149-406...</t>
+          <t>78e4167a-3b8...</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6bb8d368-ac2...</t>
+          <t>8620d797-6c7...</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1433,10 +1433,10 @@
         <v>1009532.3</v>
       </c>
       <c r="F19" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G19" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1451,12 +1451,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>31cfeff6-3d5...</t>
+          <t>e81b22a3-8bf...</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>6a0c0722-cee...</t>
+          <t>5fc0d48e-970...</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1473,10 +1473,10 @@
         <v>167097.36</v>
       </c>
       <c r="F20" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G20" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1491,12 +1491,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>f02220d1-3e5...</t>
+          <t>b5b2e52c-1d7...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>1c89880c-ce0...</t>
+          <t>8501a4bc-6d7...</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1513,10 +1513,10 @@
         <v>489746.44</v>
       </c>
       <c r="F21" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G21" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1531,12 +1531,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>b0d99f5e-a38...</t>
+          <t>9d9e7159-064...</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>fc902cab-252...</t>
+          <t>5bb27b63-b36...</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1553,10 +1553,10 @@
         <v>4430054.25</v>
       </c>
       <c r="F22" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G22" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1571,12 +1571,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>1b6d6f9a-d05...</t>
+          <t>55af06d3-cc1...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>628f5492-681...</t>
+          <t>7227ae7b-d65...</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1593,10 +1593,10 @@
         <v>106667.98</v>
       </c>
       <c r="F23" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G23" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1611,12 +1611,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>1bac2a15-e99...</t>
+          <t>7d87f682-791...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>69d7fa10-b77...</t>
+          <t>6965c103-8e7...</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1633,10 +1633,10 @@
         <v>218610</v>
       </c>
       <c r="F24" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G24" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1651,12 +1651,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>506037f5-927...</t>
+          <t>70696942-e01...</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d8a0979b-c49...</t>
+          <t>bcc73c78-48c...</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1673,10 +1673,10 @@
         <v>17080.64</v>
       </c>
       <c r="F25" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G25" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1691,12 +1691,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2685a404-0cd...</t>
+          <t>6e85d473-f25...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>451668af-882...</t>
+          <t>c86d07c9-37a...</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1713,10 +1713,10 @@
         <v>1467133.56</v>
       </c>
       <c r="F26" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G26" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1731,12 +1731,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ff5479b8-c0c...</t>
+          <t>ae0d74f3-957...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>bf479583-e28...</t>
+          <t>5ed9147d-69b...</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1753,10 +1753,10 @@
         <v>2591344.71</v>
       </c>
       <c r="F27" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G27" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1771,12 +1771,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>fd8c10c2-dfd...</t>
+          <t>61eb00cb-3ea...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6988e30a-d9b...</t>
+          <t>9c09bf11-111...</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1793,10 +1793,10 @@
         <v>1283606.87</v>
       </c>
       <c r="F28" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G28" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1811,12 +1811,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>06cf66f4-03e...</t>
+          <t>48d6f16f-596...</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>19039fac-c81...</t>
+          <t>2b1581a4-d75...</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1833,10 +1833,10 @@
         <v>668050.47</v>
       </c>
       <c r="F29" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G29" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1851,12 +1851,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>f24bb6e9-625...</t>
+          <t>b81f85e1-111...</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>5589fb8d-fce...</t>
+          <t>0d539ae6-e26...</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1873,10 +1873,10 @@
         <v>19095</v>
       </c>
       <c r="F30" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G30" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1891,12 +1891,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>a55288ab-b0c...</t>
+          <t>220e449e-04c...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>1c621a9c-34f...</t>
+          <t>936db568-381...</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1913,10 +1913,10 @@
         <v>16159.74</v>
       </c>
       <c r="F31" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G31" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1931,12 +1931,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ad2dcb07-cdc...</t>
+          <t>15d08cd1-a82...</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>eb30c1f2-396...</t>
+          <t>efc9fef5-6ce...</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1953,10 +1953,10 @@
         <v>13292.42</v>
       </c>
       <c r="F32" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G32" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1971,12 +1971,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2c880fff-3ba...</t>
+          <t>1454b224-112...</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>417c124b-a26...</t>
+          <t>0ac15c51-bbe...</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1993,10 +1993,10 @@
         <v>220374.84</v>
       </c>
       <c r="F33" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G33" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2011,12 +2011,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>c1d38311-ade...</t>
+          <t>a316b500-e9d...</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>8721ccaa-fae...</t>
+          <t>76d709f3-e24...</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2033,10 +2033,10 @@
         <v>2183.8</v>
       </c>
       <c r="F34" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G34" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2051,12 +2051,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>86e1f41e-5f2...</t>
+          <t>93b67a12-865...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>83e27367-677...</t>
+          <t>e735b825-9fd...</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2073,10 +2073,10 @@
         <v>20240.54</v>
       </c>
       <c r="F35" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G35" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2091,12 +2091,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2d1a6de5-569...</t>
+          <t>8a9c8004-5f3...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>8a9ba73d-41a...</t>
+          <t>13ac84d9-a1a...</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2113,10 +2113,10 @@
         <v>5933719</v>
       </c>
       <c r="F36" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G36" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2131,12 +2131,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>c9010d4d-cde...</t>
+          <t>e14b6dda-68c...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>d3638e27-912...</t>
+          <t>b7dfa65e-8d9...</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2153,10 +2153,10 @@
         <v>124378.19</v>
       </c>
       <c r="F37" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G37" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2171,12 +2171,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>46af92ff-44a...</t>
+          <t>93169a8c-1cb...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>500cc426-2e0...</t>
+          <t>3d14e340-abe...</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2193,10 +2193,10 @@
         <v>186285.88</v>
       </c>
       <c r="F38" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G38" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2211,12 +2211,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>96e9747f-8c6...</t>
+          <t>863b2d0b-2a9...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ba927df2-a27...</t>
+          <t>f0f077c1-9b4...</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2233,10 +2233,10 @@
         <v>433884.36</v>
       </c>
       <c r="F39" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G39" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2251,12 +2251,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>8cb62bee-3c8...</t>
+          <t>bd356244-273...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>f21aa8d8-c00...</t>
+          <t>fe46d079-b37...</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2273,10 +2273,10 @@
         <v>29162.31</v>
       </c>
       <c r="F40" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G40" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2291,12 +2291,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>e0b807b0-d16...</t>
+          <t>27a59a30-120...</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>60b72044-63e...</t>
+          <t>85f72ada-512...</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2313,10 +2313,10 @@
         <v>5352106.44</v>
       </c>
       <c r="F41" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G41" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2331,12 +2331,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>73610237-43e...</t>
+          <t>2231bbf7-038...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>775b8f0f-e44...</t>
+          <t>96c92044-7f4...</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2353,10 +2353,10 @@
         <v>798547.12</v>
       </c>
       <c r="F42" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G42" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2371,12 +2371,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>43aeb420-f76...</t>
+          <t>4557219b-e10...</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>63357bdc-81a...</t>
+          <t>900b8e26-7e2...</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2393,10 +2393,10 @@
         <v>15204408.5</v>
       </c>
       <c r="F43" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G43" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2411,12 +2411,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>9d42ef59-d57...</t>
+          <t>d67c892f-a3f...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>2d1477b6-299...</t>
+          <t>3031dd62-7f0...</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2433,10 +2433,10 @@
         <v>485420.64</v>
       </c>
       <c r="F44" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G44" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2451,12 +2451,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>a1cbab0f-39f...</t>
+          <t>2bd69ec4-a0c...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>44525171-0d5...</t>
+          <t>65f2aa78-5f7...</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2473,10 +2473,10 @@
         <v>117113.38</v>
       </c>
       <c r="F45" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G45" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2491,12 +2491,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>5b106e07-74d...</t>
+          <t>60865863-892...</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>38df8418-238...</t>
+          <t>6f6d7d38-eb1...</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2513,10 +2513,10 @@
         <v>2281177.44</v>
       </c>
       <c r="F46" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G46" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2531,12 +2531,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>a1b99081-1ef...</t>
+          <t>6bd5bb64-1a8...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>5d4419ae-390...</t>
+          <t>be8da86e-6cf...</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2553,10 +2553,10 @@
         <v>454634.51</v>
       </c>
       <c r="F47" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G47" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2571,12 +2571,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>13c63933-c9c...</t>
+          <t>6e07ed21-6da...</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>df9d8810-7c9...</t>
+          <t>94bf958c-d2f...</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2593,10 +2593,10 @@
         <v>130614.02</v>
       </c>
       <c r="F48" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G48" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -2611,12 +2611,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>899d2c66-7fb...</t>
+          <t>8aade65f-3e4...</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>3c34df29-c21...</t>
+          <t>7346af3b-d45...</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2633,10 +2633,10 @@
         <v>9379985.6</v>
       </c>
       <c r="F49" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G49" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2651,12 +2651,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>93f8495d-abf...</t>
+          <t>5c014ae1-57f...</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>65ea6e3a-c6b...</t>
+          <t>d46b1edc-f64...</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2673,10 +2673,10 @@
         <v>200038.95</v>
       </c>
       <c r="F50" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G50" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2691,12 +2691,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>f09ac7a7-8e6...</t>
+          <t>74739f2c-22c...</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>f2e8c188-842...</t>
+          <t>3300750b-ca3...</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2713,10 +2713,10 @@
         <v>5578236.3</v>
       </c>
       <c r="F51" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G51" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2731,12 +2731,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>313e2660-15f...</t>
+          <t>6bb84948-eb9...</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>b570b728-1d7...</t>
+          <t>33f27a79-dd8...</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2753,10 +2753,10 @@
         <v>384635.2</v>
       </c>
       <c r="F52" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G52" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2771,12 +2771,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>71ffbf04-899...</t>
+          <t>f6aef656-d81...</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>2ac67a29-c27...</t>
+          <t>27f88747-09b...</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2793,10 +2793,10 @@
         <v>966183.37</v>
       </c>
       <c r="F53" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G53" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2811,12 +2811,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>a4a2d1c6-cbd...</t>
+          <t>af049e96-eea...</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>e7db7a5f-444...</t>
+          <t>54dfba69-721...</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2833,10 +2833,10 @@
         <v>2661040.96</v>
       </c>
       <c r="F54" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G54" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2851,12 +2851,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>3c45112b-f00...</t>
+          <t>08e2cece-3e5...</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>1c5352ef-070...</t>
+          <t>6a3ccab6-103...</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2873,10 +2873,10 @@
         <v>141585.05</v>
       </c>
       <c r="F55" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G55" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2891,12 +2891,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>81cd2923-db5...</t>
+          <t>d4860cef-f3f...</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>596ab486-225...</t>
+          <t>03649c3d-b3d...</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2913,10 +2913,10 @@
         <v>43232.28</v>
       </c>
       <c r="F56" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G56" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2931,12 +2931,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>4e3992b5-8c5...</t>
+          <t>cd717ae4-f1b...</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>49889448-f20...</t>
+          <t>36b14fff-921...</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2953,10 +2953,10 @@
         <v>314796.5</v>
       </c>
       <c r="F57" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G57" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -2971,12 +2971,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>6539310d-9ce...</t>
+          <t>3f19c84d-c72...</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>74f4e4cf-494...</t>
+          <t>0be0d979-3a3...</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2993,10 +2993,10 @@
         <v>2000761.71</v>
       </c>
       <c r="F58" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G58" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3011,12 +3011,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>5b9e5f04-346...</t>
+          <t>95158766-96e...</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>705f8238-7e3...</t>
+          <t>4fc50bc6-8f5...</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3033,10 +3033,10 @@
         <v>492.67</v>
       </c>
       <c r="F59" t="n">
-        <v>-19</v>
+        <v>-21</v>
       </c>
       <c r="G59" t="n">
-        <v>-449.7</v>
+        <v>-502.8</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>018895fb-d4d...</t>
+          <t>9ade513a-1a4...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5266,7 +5266,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>78fdc73f-d4f...</t>
+          <t>b91a1ee6-bd9...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>f95abe04-343...</t>
+          <t>8984e90d-58e...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>

<commit_message>
Update generated settlement reports from latest pipeline run
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/generated/settlement_report.xlsx
+++ b/data/generated/settlement_report.xlsx
@@ -494,7 +494,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-06-23 23:53</t>
+          <t>2026-06-24 00:10</t>
         </is>
       </c>
     </row>
@@ -731,12 +731,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>37e29856-a68...</t>
+          <t>004bd2c6-4e6...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>95b14ee7-93c...</t>
+          <t>1ca1e7dd-15e...</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -756,7 +756,7 @@
         <v>-22</v>
       </c>
       <c r="G2" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H2" t="inlineStr">
         <is>
@@ -771,12 +771,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>bd59965b-f20...</t>
+          <t>61c436ac-384...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>8c0295a9-bfe...</t>
+          <t>8d9e5cf6-2db...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -796,7 +796,7 @@
         <v>-22</v>
       </c>
       <c r="G3" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -811,12 +811,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3e1c6b78-3ed...</t>
+          <t>82d58827-edf...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>22dc9aae-7c5...</t>
+          <t>3946ee01-4c1...</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -836,7 +836,7 @@
         <v>-22</v>
       </c>
       <c r="G4" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -851,12 +851,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>fbf322a7-2d9...</t>
+          <t>d5312b9e-707...</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>da648678-1e6...</t>
+          <t>e6e18357-e89...</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -876,7 +876,7 @@
         <v>-22</v>
       </c>
       <c r="G5" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -891,12 +891,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ac9aaaca-4be...</t>
+          <t>15f5439e-19a...</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>4dee1125-e3c...</t>
+          <t>d299a1ee-a9a...</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -916,7 +916,7 @@
         <v>-22</v>
       </c>
       <c r="G6" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -931,12 +931,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>744e454f-2fc...</t>
+          <t>7714a5f1-81f...</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>f7f29f94-26e...</t>
+          <t>a23ac16b-6c1...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -956,7 +956,7 @@
         <v>-22</v>
       </c>
       <c r="G7" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -971,12 +971,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>b9f7d250-68a...</t>
+          <t>94a0e7c6-f81...</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>b08516d8-f18...</t>
+          <t>777b2053-da6...</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -996,7 +996,7 @@
         <v>-22</v>
       </c>
       <c r="G8" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1011,12 +1011,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>90e8bb8a-801...</t>
+          <t>0d1f08d7-662...</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>d7905644-0ec...</t>
+          <t>d64ce261-f85...</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1036,7 +1036,7 @@
         <v>-22</v>
       </c>
       <c r="G9" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1051,12 +1051,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>035c98ab-f80...</t>
+          <t>63bffa20-401...</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>167d5848-620...</t>
+          <t>768c62f3-ac0...</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1076,7 +1076,7 @@
         <v>-22</v>
       </c>
       <c r="G10" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
@@ -1091,12 +1091,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>e8f7eb38-0fa...</t>
+          <t>05c2c80c-ad9...</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>52f8600a-dfe...</t>
+          <t>aa4906f2-a0c...</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1116,7 +1116,7 @@
         <v>-22</v>
       </c>
       <c r="G11" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1131,12 +1131,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>05f7fb87-d02...</t>
+          <t>ccbb3b0f-6bc...</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>9881cb09-c7b...</t>
+          <t>2a4ca1e1-76e...</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1156,7 +1156,7 @@
         <v>-22</v>
       </c>
       <c r="G12" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1171,12 +1171,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>c3288b65-2f9...</t>
+          <t>ad51150e-a96...</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5cb2e45b-f28...</t>
+          <t>94d34494-934...</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1196,7 +1196,7 @@
         <v>-22</v>
       </c>
       <c r="G13" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
@@ -1211,12 +1211,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>18d39dd6-399...</t>
+          <t>c0da7d50-f11...</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>73fff836-7cf...</t>
+          <t>a9b3df27-d10...</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1236,7 +1236,7 @@
         <v>-22</v>
       </c>
       <c r="G14" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1251,12 +1251,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>4f716abf-616...</t>
+          <t>aeed7578-0c8...</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>c28fe5a9-eb8...</t>
+          <t>3bb0b899-955...</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1276,7 +1276,7 @@
         <v>-22</v>
       </c>
       <c r="G15" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
@@ -1291,12 +1291,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2c329023-dad...</t>
+          <t>1aabe09e-ba7...</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>69798e2c-49f...</t>
+          <t>9c302ece-f79...</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1316,7 +1316,7 @@
         <v>-22</v>
       </c>
       <c r="G16" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
@@ -1331,12 +1331,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2dae8e06-624...</t>
+          <t>91fcaf4e-4dd...</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>735c7992-9bd...</t>
+          <t>ce930d68-a31...</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -1356,7 +1356,7 @@
         <v>-22</v>
       </c>
       <c r="G17" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
@@ -1371,12 +1371,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>6d0f40c1-016...</t>
+          <t>75bfa8b2-6fb...</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>d438a187-5de...</t>
+          <t>b4007144-009...</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1396,7 +1396,7 @@
         <v>-22</v>
       </c>
       <c r="G18" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -1411,12 +1411,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>3ed77df0-54d...</t>
+          <t>66224b2b-41f...</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>85bf61c9-ee2...</t>
+          <t>fa0f64f6-b36...</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1436,7 +1436,7 @@
         <v>-22</v>
       </c>
       <c r="G19" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
@@ -1451,12 +1451,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>cc80fc8a-773...</t>
+          <t>fe48aa82-2c8...</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>b072b5fa-839...</t>
+          <t>08cd28f8-4c2...</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1476,7 +1476,7 @@
         <v>-22</v>
       </c>
       <c r="G20" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
@@ -1491,12 +1491,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>32bf868e-c4e...</t>
+          <t>8a3aaf5c-d01...</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>64065349-89f...</t>
+          <t>5d2bef27-f70...</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1516,7 +1516,7 @@
         <v>-22</v>
       </c>
       <c r="G21" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
@@ -1531,12 +1531,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>57827612-f95...</t>
+          <t>d066ffce-526...</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>077f922e-8b7...</t>
+          <t>ae802ca2-0d7...</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1556,7 +1556,7 @@
         <v>-22</v>
       </c>
       <c r="G22" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
@@ -1571,12 +1571,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>8ca9b85b-5e3...</t>
+          <t>604e6e52-48a...</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>52de0937-e33...</t>
+          <t>c2d0b0df-ee5...</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -1596,7 +1596,7 @@
         <v>-22</v>
       </c>
       <c r="G23" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H23" t="inlineStr">
         <is>
@@ -1611,12 +1611,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>9e9a40d6-6cb...</t>
+          <t>faa7d523-b69...</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>14e520b0-759...</t>
+          <t>c102493e-26d...</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1636,7 +1636,7 @@
         <v>-22</v>
       </c>
       <c r="G24" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
@@ -1651,12 +1651,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>1d6dfd0e-5ad...</t>
+          <t>0be98fce-b11...</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>d6e2edab-5a3...</t>
+          <t>92fe8b15-49a...</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1676,7 +1676,7 @@
         <v>-22</v>
       </c>
       <c r="G25" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
@@ -1691,12 +1691,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>e54bae68-3dd...</t>
+          <t>a778d275-f59...</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5efd88e1-1aa...</t>
+          <t>a39daae0-c66...</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -1716,7 +1716,7 @@
         <v>-22</v>
       </c>
       <c r="G26" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
@@ -1731,12 +1731,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>a37748ce-acf...</t>
+          <t>cc55bd21-a21...</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>91dd9330-d83...</t>
+          <t>c62bf8eb-ec7...</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -1756,7 +1756,7 @@
         <v>-22</v>
       </c>
       <c r="G27" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
@@ -1771,12 +1771,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>1c214211-e90...</t>
+          <t>49a052cc-434...</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2b80e188-057...</t>
+          <t>399047a8-be0...</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -1796,7 +1796,7 @@
         <v>-22</v>
       </c>
       <c r="G28" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
@@ -1811,12 +1811,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>1db64b23-4c0...</t>
+          <t>7b5a2f32-ab6...</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>4ed14501-4c3...</t>
+          <t>e2617b4c-f48...</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -1836,7 +1836,7 @@
         <v>-22</v>
       </c>
       <c r="G29" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
@@ -1851,12 +1851,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>72647480-278...</t>
+          <t>babaf211-842...</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2fafd403-240...</t>
+          <t>db73f4b2-b0c...</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -1876,7 +1876,7 @@
         <v>-22</v>
       </c>
       <c r="G30" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
@@ -1891,12 +1891,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>e2e2aeb3-8fa...</t>
+          <t>a18bd69d-c42...</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>0e06876f-cdd...</t>
+          <t>b8db72f5-0ee...</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1916,7 +1916,7 @@
         <v>-22</v>
       </c>
       <c r="G31" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -1931,12 +1931,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2cef3717-af3...</t>
+          <t>b918f7d2-73c...</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>f62d39f9-315...</t>
+          <t>56ff84bc-2b4...</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1956,7 +1956,7 @@
         <v>-22</v>
       </c>
       <c r="G32" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -1971,12 +1971,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>3ffe9948-f70...</t>
+          <t>50738a17-936...</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>99ba6943-9a9...</t>
+          <t>cb0c5f42-482...</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1996,7 +1996,7 @@
         <v>-22</v>
       </c>
       <c r="G33" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H33" t="inlineStr">
         <is>
@@ -2011,12 +2011,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>000a6224-7ba...</t>
+          <t>4ecb0fd4-de1...</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2679fb7f-837...</t>
+          <t>53ce1a65-bb1...</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -2036,7 +2036,7 @@
         <v>-22</v>
       </c>
       <c r="G34" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
@@ -2051,12 +2051,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>8f12d662-206...</t>
+          <t>ccb706e4-15e...</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>802d8e77-9e6...</t>
+          <t>95728acb-bc1...</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -2076,7 +2076,7 @@
         <v>-22</v>
       </c>
       <c r="G35" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -2091,12 +2091,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>fc7fa442-970...</t>
+          <t>99d9ac16-085...</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>d0bbbf30-139...</t>
+          <t>069cdbd7-ffc...</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -2116,7 +2116,7 @@
         <v>-22</v>
       </c>
       <c r="G36" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
@@ -2131,12 +2131,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>495168d3-8eb...</t>
+          <t>f1e4898d-d2a...</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>464f0813-aa0...</t>
+          <t>8a45378c-957...</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -2156,7 +2156,7 @@
         <v>-22</v>
       </c>
       <c r="G37" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H37" t="inlineStr">
         <is>
@@ -2171,12 +2171,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>4c39dd15-854...</t>
+          <t>c9d76829-f5a...</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>f966239b-7e1...</t>
+          <t>8d7aed0d-ce2...</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -2196,7 +2196,7 @@
         <v>-22</v>
       </c>
       <c r="G38" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
@@ -2211,12 +2211,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>8d54aa06-385...</t>
+          <t>1dc9f30e-4e7...</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>98bc2c61-ea0...</t>
+          <t>86940641-8cd...</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2236,7 +2236,7 @@
         <v>-22</v>
       </c>
       <c r="G39" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
@@ -2251,12 +2251,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>c9b6c241-2a1...</t>
+          <t>2e5fa386-f94...</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>e0098ee2-931...</t>
+          <t>71386dcb-0d1...</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -2276,7 +2276,7 @@
         <v>-22</v>
       </c>
       <c r="G40" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
@@ -2291,12 +2291,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>42057452-5bb...</t>
+          <t>c5fb776f-50a...</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>37880f15-502...</t>
+          <t>2af5ff7b-36b...</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2316,7 +2316,7 @@
         <v>-22</v>
       </c>
       <c r="G41" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
@@ -2331,12 +2331,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>8cce3b9b-d20...</t>
+          <t>a60c7deb-949...</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ab2ec5f0-05a...</t>
+          <t>5922b2ca-ccf...</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2356,7 +2356,7 @@
         <v>-22</v>
       </c>
       <c r="G42" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
@@ -2371,12 +2371,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>346bb1d4-502...</t>
+          <t>f162b706-230...</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>23750514-b07...</t>
+          <t>12955a61-0f4...</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2396,7 +2396,7 @@
         <v>-22</v>
       </c>
       <c r="G43" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
@@ -2411,12 +2411,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>efc54315-b93...</t>
+          <t>af0947e6-2c7...</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>a862b415-0e7...</t>
+          <t>1cfe1d12-af5...</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -2436,7 +2436,7 @@
         <v>-22</v>
       </c>
       <c r="G44" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
@@ -2451,12 +2451,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>92e6dd37-992...</t>
+          <t>2c612300-121...</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>31527644-ce4...</t>
+          <t>f87f507f-aba...</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2476,7 +2476,7 @@
         <v>-22</v>
       </c>
       <c r="G45" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
@@ -2491,12 +2491,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>43a73476-0e5...</t>
+          <t>14d07b0d-813...</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>fb8a5c29-e2f...</t>
+          <t>a747190b-ecd...</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -2516,7 +2516,7 @@
         <v>-22</v>
       </c>
       <c r="G46" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
@@ -2531,12 +2531,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>00637d30-0d4...</t>
+          <t>26953193-09a...</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>47db87fb-a9d...</t>
+          <t>db82a68f-6b1...</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -2556,7 +2556,7 @@
         <v>-22</v>
       </c>
       <c r="G47" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
@@ -2571,12 +2571,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>0ce7b267-58c...</t>
+          <t>2ee7e447-bf5...</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>24edb6fb-a07...</t>
+          <t>143b0f2c-300...</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2596,7 +2596,7 @@
         <v>-22</v>
       </c>
       <c r="G48" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -2611,12 +2611,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2acf41f7-b6d...</t>
+          <t>e5c6c5f8-873...</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>1df2b62c-eb0...</t>
+          <t>f8049e89-b24...</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2636,7 +2636,7 @@
         <v>-22</v>
       </c>
       <c r="G49" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
@@ -2651,12 +2651,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>8503e45e-0ad...</t>
+          <t>95b74898-6a4...</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>d7f8b1c8-4ce...</t>
+          <t>ff120984-540...</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2676,7 +2676,7 @@
         <v>-22</v>
       </c>
       <c r="G50" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -2691,12 +2691,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>7f9b798f-4ef...</t>
+          <t>07788a1a-c52...</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>ddc48286-af6...</t>
+          <t>6ca25c10-4bc...</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2716,7 +2716,7 @@
         <v>-22</v>
       </c>
       <c r="G51" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
@@ -2731,12 +2731,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>44781d4d-e71...</t>
+          <t>aa08a8b4-999...</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>1a578d33-a56...</t>
+          <t>d3e5c74e-f26...</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2756,7 +2756,7 @@
         <v>-22</v>
       </c>
       <c r="G52" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
@@ -2771,12 +2771,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>d5391c64-6e2...</t>
+          <t>d49a320e-ce6...</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>188dfd2c-e36...</t>
+          <t>32f19f0a-5a2...</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2796,7 +2796,7 @@
         <v>-22</v>
       </c>
       <c r="G53" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
@@ -2811,12 +2811,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>1532afef-455...</t>
+          <t>c278a38e-9f2...</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>f04bbaca-416...</t>
+          <t>389343d6-4aa...</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2836,7 +2836,7 @@
         <v>-22</v>
       </c>
       <c r="G54" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -2851,12 +2851,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>81d2f531-d54...</t>
+          <t>5454a2c0-d32...</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ae5a648d-862...</t>
+          <t>67e57d6c-d86...</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2876,7 +2876,7 @@
         <v>-22</v>
       </c>
       <c r="G55" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
@@ -2891,12 +2891,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>10bcfa6c-de0...</t>
+          <t>773e48b2-de6...</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>b8895c34-649...</t>
+          <t>c38de897-09d...</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2916,7 +2916,7 @@
         <v>-22</v>
       </c>
       <c r="G56" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
@@ -2931,12 +2931,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>62655fc2-3b8...</t>
+          <t>f0583b19-b54...</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>e32f404f-716...</t>
+          <t>57ecb82e-56f...</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2956,7 +2956,7 @@
         <v>-22</v>
       </c>
       <c r="G57" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
@@ -2971,12 +2971,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>bc2d7650-fe8...</t>
+          <t>3326d090-97e...</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>b3402667-5ef...</t>
+          <t>8bd9b946-7dd...</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -2996,7 +2996,7 @@
         <v>-22</v>
       </c>
       <c r="G58" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3011,12 +3011,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>c8aa6ee0-045...</t>
+          <t>598fd364-b64...</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>412ebd2c-e7e...</t>
+          <t>eddbb857-db6...</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -3036,7 +3036,7 @@
         <v>-22</v>
       </c>
       <c r="G59" t="n">
-        <v>-509.9</v>
+        <v>-510.2</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
@@ -5227,7 +5227,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>e5414b28-24f...</t>
+          <t>ea70b0b6-a37...</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -5266,7 +5266,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>fba0fc56-e85...</t>
+          <t>5898e926-86e...</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -5305,7 +5305,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>89e5a342-a8a...</t>
+          <t>c5904691-337...</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">

</xml_diff>